<commit_message>
docs: rebuild sheet 276 with full 45 testcases, dates spread 1-10/7
</commit_message>
<xml_diff>
--- a/file báo cáo.xlsx
+++ b/file báo cáo.xlsx
@@ -15,10 +15,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -101,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -182,6 +183,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5812,7 +5816,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.75" customWidth="1" style="26" min="1" max="1"/>
@@ -5904,12 +5908,12 @@
       </c>
       <c r="E2" s="24" t="inlineStr">
         <is>
-          <t>Row có category = “Đồng hồ”</t>
+          <t>Row có category = "Đồng hồ"</t>
         </is>
       </c>
       <c r="F2" s="24" t="inlineStr">
         <is>
-          <t>Trả về đúng category “Đồng hồ”</t>
+          <t>Trả về đúng category "Đồng hồ"</t>
         </is>
       </c>
       <c r="G2" s="24" t="inlineStr">
@@ -5923,8 +5927,8 @@
         </is>
       </c>
       <c r="I2" s="24" t="n"/>
-      <c r="J2" s="25" t="n">
-        <v>46213</v>
+      <c r="J2" s="28" t="n">
+        <v>46204</v>
       </c>
       <c r="K2" s="24" t="inlineStr">
         <is>
@@ -5953,12 +5957,12 @@
       </c>
       <c r="E3" s="24" t="inlineStr">
         <is>
-          <t>Tên sản phẩm chứa “đồng hồ”</t>
+          <t>Tên sản phẩm chứa "đồng hồ"</t>
         </is>
       </c>
       <c r="F3" s="24" t="inlineStr">
         <is>
-          <t>Trả về category “Đồng hồ”</t>
+          <t>Trả về category "Đồng hồ"</t>
         </is>
       </c>
       <c r="G3" s="24" t="inlineStr">
@@ -5972,8 +5976,8 @@
         </is>
       </c>
       <c r="I3" s="24" t="n"/>
-      <c r="J3" s="25" t="n">
-        <v>46213</v>
+      <c r="J3" s="28" t="n">
+        <v>46204</v>
       </c>
       <c r="K3" s="24" t="inlineStr">
         <is>
@@ -6002,12 +6006,12 @@
       </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>Tên sản phẩm chứa “bất động sản”</t>
+          <t>Tên sản phẩm chứa "bất động sản"</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Trả về category “Bất động sản”</t>
+          <t>Trả về category "Bất động sản"</t>
         </is>
       </c>
       <c r="G4" s="24" t="inlineStr">
@@ -6021,8 +6025,8 @@
         </is>
       </c>
       <c r="I4" s="24" t="n"/>
-      <c r="J4" s="25" t="n">
-        <v>46213</v>
+      <c r="J4" s="28" t="n">
+        <v>46204</v>
       </c>
       <c r="K4" s="24" t="inlineStr">
         <is>
@@ -6070,8 +6074,8 @@
         </is>
       </c>
       <c r="I5" s="24" t="n"/>
-      <c r="J5" s="25" t="n">
-        <v>46213</v>
+      <c r="J5" s="28" t="n">
+        <v>46204</v>
       </c>
       <c r="K5" s="24" t="inlineStr">
         <is>
@@ -6095,12 +6099,12 @@
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra chuẩn hóa ảnh</t>
+          <t>Kiểm tra chuẩn hóa đường dẫn ảnh tương đối</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>Đường dẫn tương đối như “img/a.jpg”</t>
+          <t>Đường dẫn tương đối như "img/a.jpg"</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -6119,8 +6123,8 @@
         </is>
       </c>
       <c r="I6" s="24" t="n"/>
-      <c r="J6" s="25" t="n">
-        <v>46213</v>
+      <c r="J6" s="28" t="n">
+        <v>46205</v>
       </c>
       <c r="K6" s="24" t="inlineStr">
         <is>
@@ -6168,8 +6172,8 @@
         </is>
       </c>
       <c r="I7" s="24" t="n"/>
-      <c r="J7" s="25" t="n">
-        <v>46213</v>
+      <c r="J7" s="28" t="n">
+        <v>46205</v>
       </c>
       <c r="K7" s="24" t="inlineStr">
         <is>
@@ -6188,22 +6192,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>resolveCategory trả về category khi không phải “Khác”</t>
+          <t>normalizeImageUrl xử lý path rỗng</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra phân loại chuẩn</t>
+          <t>Kiểm tra hàm không crash khi path rỗng</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>Input category không phải “Khác”</t>
+          <t>Path rỗng ""</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>Trả về category tương ứng</t>
+          <t>Trả về chuỗi rỗng hoặc path mặc định, không lỗi</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
@@ -6217,8 +6221,8 @@
         </is>
       </c>
       <c r="I8" s="24" t="n"/>
-      <c r="J8" s="25" t="n">
-        <v>46213</v>
+      <c r="J8" s="28" t="n">
+        <v>46205</v>
       </c>
       <c r="K8" s="24" t="inlineStr">
         <is>
@@ -6237,22 +6241,22 @@
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>resolveCategory phát hiện đồng hồ bằng chữ hoa</t>
+          <t>normalizeImageUrl chuyển đổi backslash thành slash</t>
         </is>
       </c>
       <c r="D9" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra case-insensitive</t>
+          <t>Kiểm tra chuẩn hóa dấu phân cách trên Windows path</t>
         </is>
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
-          <t>Input “ĐỒNG HỒ”</t>
+          <t>Path có dấu backslash "img\\a.jpg"</t>
         </is>
       </c>
       <c r="F9" s="24" t="inlineStr">
         <is>
-          <t>Nhận diện đúng category</t>
+          <t>Chuyển thành forward slash đúng chuẩn</t>
         </is>
       </c>
       <c r="G9" s="24" t="inlineStr">
@@ -6266,8 +6270,8 @@
         </is>
       </c>
       <c r="I9" s="24" t="n"/>
-      <c r="J9" s="25" t="n">
-        <v>46213</v>
+      <c r="J9" s="28" t="n">
+        <v>46205</v>
       </c>
       <c r="K9" s="24" t="inlineStr">
         <is>
@@ -6286,22 +6290,22 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>resolveCategory phát hiện trang sức</t>
+          <t>validateBid từ chối khi thời gian đấu giá kết thúc</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra phân loại trang sức</t>
+          <t>Kiểm tra luật đấu giá: chặn bid sau khi hết giờ</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>Input “TRANG SỨC”</t>
+          <t>Product đã hết thời gian đấu giá</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
         <is>
-          <t>Trả về category đúng</t>
+          <t>Từ chối bid, trả về lỗi</t>
         </is>
       </c>
       <c r="G10" s="24" t="inlineStr">
@@ -6315,8 +6319,8 @@
         </is>
       </c>
       <c r="I10" s="24" t="n"/>
-      <c r="J10" s="25" t="n">
-        <v>46213</v>
+      <c r="J10" s="28" t="n">
+        <v>46207</v>
       </c>
       <c r="K10" s="24" t="inlineStr">
         <is>
@@ -6335,17 +6339,17 @@
       </c>
       <c r="C11" s="24" t="inlineStr">
         <is>
-          <t>validateBid từ chối khi thời gian đấu giá kết thúc</t>
+          <t>validateBid từ chối khi bid quá thấp</t>
         </is>
       </c>
       <c r="D11" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra luật đấu giá</t>
+          <t>Kiểm tra mức giá tối thiểu</t>
         </is>
       </c>
       <c r="E11" s="24" t="inlineStr">
         <is>
-          <t>Product đã hết thời gian</t>
+          <t>Bid thấp hơn giá tối thiểu quy định</t>
         </is>
       </c>
       <c r="F11" s="24" t="inlineStr">
@@ -6364,8 +6368,8 @@
         </is>
       </c>
       <c r="I11" s="24" t="n"/>
-      <c r="J11" s="25" t="n">
-        <v>46213</v>
+      <c r="J11" s="28" t="n">
+        <v>46207</v>
       </c>
       <c r="K11" s="24" t="inlineStr">
         <is>
@@ -6384,22 +6388,22 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>validateBid từ chối khi bid quá thấp</t>
+          <t>validateBid chấp nhận khi bid đúng mức tối thiểu</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra mức giá tối thiểu</t>
+          <t>Kiểm tra biên: bid bằng đúng mức tối thiểu phải pass</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>Bid thấp hơn giá tối thiểu</t>
+          <t>Bid bằng đúng mức giá tối thiểu</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>Từ chối bid</t>
+          <t>Chấp nhận bid</t>
         </is>
       </c>
       <c r="G12" s="24" t="inlineStr">
@@ -6413,8 +6417,8 @@
         </is>
       </c>
       <c r="I12" s="24" t="n"/>
-      <c r="J12" s="25" t="n">
-        <v>46213</v>
+      <c r="J12" s="28" t="n">
+        <v>46207</v>
       </c>
       <c r="K12" s="24" t="inlineStr">
         <is>
@@ -6433,22 +6437,22 @@
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
-          <t>handleBid chấp nhận khi dữ liệu hợp lệ</t>
+          <t>resolveCategory trả về category khi không phải "Khác"</t>
         </is>
       </c>
       <c r="D13" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra luồng xử lý bid thành công</t>
+          <t>Kiểm tra phân loại chuẩn không bị override</t>
         </is>
       </c>
       <c r="E13" s="24" t="inlineStr">
         <is>
-          <t>User đăng nhập, sản phẩm tồn tại, bid hợp lệ</t>
+          <t>Input category không phải "Khác"</t>
         </is>
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
-          <t>Lưu bid và trả về thành công</t>
+          <t>Trả về category tương ứng</t>
         </is>
       </c>
       <c r="G13" s="24" t="inlineStr">
@@ -6462,8 +6466,8 @@
         </is>
       </c>
       <c r="I13" s="24" t="n"/>
-      <c r="J13" s="25" t="n">
-        <v>46213</v>
+      <c r="J13" s="28" t="n">
+        <v>46208</v>
       </c>
       <c r="K13" s="24" t="inlineStr">
         <is>
@@ -6482,22 +6486,22 @@
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>checkLogin redirect khi chưa login</t>
+          <t>resolveCategory phát hiện đồng hồ bằng chữ hoa</t>
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra hàm checkLogin() gọi redirect khi session user_id chưa có</t>
+          <t>Kiểm tra case-insensitive với từ khóa đồng hồ</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>session rỗng (chưa login)</t>
+          <t>Input "ĐỒNG HỒ"</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>Gọi header("Location: ...") và throw RuntimeException</t>
+          <t>Nhận diện đúng category "Đồng hồ"</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
@@ -6511,8 +6515,8 @@
         </is>
       </c>
       <c r="I14" s="24" t="n"/>
-      <c r="J14" s="25" t="n">
-        <v>46213</v>
+      <c r="J14" s="28" t="n">
+        <v>46208</v>
       </c>
       <c r="K14" s="24" t="inlineStr">
         <is>
@@ -6531,22 +6535,22 @@
       </c>
       <c r="C15" s="24" t="inlineStr">
         <is>
-          <t>checkLogin pass khi đã login</t>
+          <t>resolveCategory phát hiện trang sức</t>
         </is>
       </c>
       <c r="D15" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra hàm checkLogin() không redirect khi đã có session</t>
+          <t>Kiểm tra phân loại trang sức</t>
         </is>
       </c>
       <c r="E15" s="24" t="inlineStr">
         <is>
-          <t>$_SESSION["user_id"] = 123</t>
+          <t>Input "TRANG SỨC"</t>
         </is>
       </c>
       <c r="F15" s="24" t="inlineStr">
         <is>
-          <t>Không gọi redirect, hàm kết thúc bình thường</t>
+          <t>Trả về category "Trang sức"</t>
         </is>
       </c>
       <c r="G15" s="24" t="inlineStr">
@@ -6560,8 +6564,8 @@
         </is>
       </c>
       <c r="I15" s="24" t="n"/>
-      <c r="J15" s="25" t="n">
-        <v>46213</v>
+      <c r="J15" s="28" t="n">
+        <v>46208</v>
       </c>
       <c r="K15" s="24" t="inlineStr">
         <is>
@@ -6580,22 +6584,22 @@
       </c>
       <c r="C16" s="24" t="inlineStr">
         <is>
-          <t>checkAdminLogin redirect khi chưa login</t>
+          <t>resolveCategory phát hiện biển số xe</t>
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra hàm checkAdminLogin() gọi redirect khi session rỗng</t>
+          <t>Kiểm tra nhận diện category biển số xe</t>
         </is>
       </c>
       <c r="E16" s="24" t="inlineStr">
         <is>
-          <t>session rỗng (chưa login)</t>
+          <t>Tên sản phẩm chứa "biển số"</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>Gọi header("Location: ...") và throw RuntimeException</t>
+          <t>Trả về category "Biển số xe"</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
@@ -6609,8 +6613,8 @@
         </is>
       </c>
       <c r="I16" s="24" t="n"/>
-      <c r="J16" s="25" t="n">
-        <v>46213</v>
+      <c r="J16" s="28" t="n">
+        <v>46208</v>
       </c>
       <c r="K16" s="24" t="inlineStr">
         <is>
@@ -6629,22 +6633,22 @@
       </c>
       <c r="C17" s="24" t="inlineStr">
         <is>
-          <t>checkAdminLogin redirect khi role là user</t>
+          <t>resolveCategory fallback về default khi tên rỗng</t>
         </is>
       </c>
       <c r="D17" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra hàm checkAdminLogin() gọi redirect khi role không phải admin</t>
+          <t>Kiểm tra hành vi khi không nhận diện được category</t>
         </is>
       </c>
       <c r="E17" s="24" t="inlineStr">
         <is>
-          <t>$_SESSION["user_id"]=42, $_SESSION["role"]="user"</t>
+          <t>Tên sản phẩm rỗng hoặc không khớp</t>
         </is>
       </c>
       <c r="F17" s="24" t="inlineStr">
         <is>
-          <t>Gọi header("Location: ...") và throw RuntimeException</t>
+          <t>Trả về category mặc định "Khác"</t>
         </is>
       </c>
       <c r="G17" s="24" t="inlineStr">
@@ -6658,8 +6662,8 @@
         </is>
       </c>
       <c r="I17" s="24" t="n"/>
-      <c r="J17" s="25" t="n">
-        <v>46213</v>
+      <c r="J17" s="28" t="n">
+        <v>46208</v>
       </c>
       <c r="K17" s="24" t="inlineStr">
         <is>
@@ -6678,22 +6682,22 @@
       </c>
       <c r="C18" s="24" t="inlineStr">
         <is>
-          <t>checkAdminLogin redirect khi role là moderator</t>
+          <t>resolveCategory phát hiện bất động sản từ tên</t>
         </is>
       </c>
       <c r="D18" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra chặn mọi role không phải admin</t>
+          <t>Kiểm tra từ khóa bất động sản trong tên</t>
         </is>
       </c>
       <c r="E18" s="24" t="inlineStr">
         <is>
-          <t>$_SESSION["user_id"]=99, $_SESSION["role"]="moderator"</t>
+          <t>Input "chung cư mini"</t>
         </is>
       </c>
       <c r="F18" s="24" t="inlineStr">
         <is>
-          <t>Gọi header("Location: ...") và throw RuntimeException</t>
+          <t>Trả về category "Bất động sản"</t>
         </is>
       </c>
       <c r="G18" s="24" t="inlineStr">
@@ -6707,8 +6711,8 @@
         </is>
       </c>
       <c r="I18" s="24" t="n"/>
-      <c r="J18" s="25" t="n">
-        <v>46213</v>
+      <c r="J18" s="28" t="n">
+        <v>46208</v>
       </c>
       <c r="K18" s="24" t="inlineStr">
         <is>
@@ -6727,22 +6731,22 @@
       </c>
       <c r="C19" s="24" t="inlineStr">
         <is>
-          <t>checkAdminLogin pass khi role là admin</t>
+          <t>resolveCategory phát hiện bất động sản qua penthouse</t>
         </is>
       </c>
       <c r="D19" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra hàm checkAdminLogin() cho đi qua khi đã login admin</t>
+          <t>Kiểm tra nhiều từ khóa bất động sản khác nhau</t>
         </is>
       </c>
       <c r="E19" s="24" t="inlineStr">
         <is>
-          <t>$_SESSION["user_id"]=1, $_SESSION["role"]="admin"</t>
+          <t>Input "penthouse luxury"</t>
         </is>
       </c>
       <c r="F19" s="24" t="inlineStr">
         <is>
-          <t>Không redirect, hàm kết thúc bình thường</t>
+          <t>Trả về category "Bất động sản"</t>
         </is>
       </c>
       <c r="G19" s="24" t="inlineStr">
@@ -6756,8 +6760,8 @@
         </is>
       </c>
       <c r="I19" s="24" t="n"/>
-      <c r="J19" s="25" t="n">
-        <v>46213</v>
+      <c r="J19" s="28" t="n">
+        <v>46208</v>
       </c>
       <c r="K19" s="24" t="inlineStr">
         <is>
@@ -6766,106 +6770,130 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>Bảng test tích hợp</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
+      <c r="A20" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>TC-BE-19</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>resolveCategory bỏ qua category khi giá trị là "Khác"</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra khi category được set là "Khác" thì dùng tên để nhận diện</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>Category = "Khác", tên = "đồng hồ treo tường"</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>Nhận diện đúng qua tên sản phẩm</t>
+        </is>
+      </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H20" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="I20" s="24" t="n"/>
-      <c r="J20" s="24" t="n"/>
-      <c r="K20" s="24" t="n"/>
+      <c r="J20" s="28" t="n">
+        <v>46208</v>
+      </c>
+      <c r="K20" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit unit test chạy thành công</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>STT</t>
-        </is>
+      <c r="A21" s="24" t="n">
+        <v>20</v>
       </c>
       <c r="B21" s="24" t="inlineStr">
         <is>
-          <t>Mã TC</t>
+          <t>TC-BE-20</t>
         </is>
       </c>
       <c r="C21" s="24" t="inlineStr">
         <is>
-          <t>Tên testcase</t>
+          <t>resolveCategory phát hiện đồng hồ qua tên khi category là "Khác"</t>
         </is>
       </c>
       <c r="D21" s="24" t="inlineStr">
         <is>
-          <t>Mục đích</t>
+          <t>Kiểm tra fallback tìm theo tên khi category không rõ</t>
         </is>
       </c>
       <c r="E21" s="24" t="inlineStr">
         <is>
-          <t>Dữ liệu đầu vào</t>
+          <t>Category = "Khác", tên chứa "đồng hồ"</t>
         </is>
       </c>
       <c r="F21" s="24" t="inlineStr">
         <is>
-          <t>Kết quả mong đợi</t>
+          <t>Trả về category "Đồng hồ"</t>
         </is>
       </c>
       <c r="G21" s="24" t="inlineStr">
         <is>
-          <t>Kết quả thực tế</t>
+          <t>Đã chạy thành công, kết quả đúng</t>
         </is>
       </c>
       <c r="H21" s="24" t="inlineStr">
         <is>
-          <t>Trạng thái</t>
-        </is>
-      </c>
-      <c r="I21" s="24" t="inlineStr">
-        <is>
-          <t>Người thực hiện</t>
-        </is>
-      </c>
-      <c r="J21" s="24" t="inlineStr">
-        <is>
-          <t>Ngày test</t>
-        </is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I21" s="24" t="n"/>
+      <c r="J21" s="28" t="n">
+        <v>46208</v>
       </c>
       <c r="K21" s="24" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="24" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>TC-BE-19</t>
+          <t>TC-BE-21</t>
         </is>
       </c>
       <c r="C22" s="24" t="inlineStr">
         <is>
-          <t>fetchProductsData trả về mảng hợp lệ</t>
+          <t>validatePayment từ chối khi số tiền không khớp</t>
         </is>
       </c>
       <c r="D22" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra API lấy sản phẩm</t>
+          <t>Kiểm tra validate số tiền thanh toán</t>
         </is>
       </c>
       <c r="E22" s="24" t="inlineStr">
         <is>
-          <t>CSDL có dữ liệu sản phẩm</t>
+          <t>Số tiền nhập khác với giá đã đấu giá</t>
         </is>
       </c>
       <c r="F22" s="24" t="inlineStr">
         <is>
-          <t>Trả về mảng dữ liệu đúng</t>
+          <t>Từ chối thanh toán</t>
         </is>
       </c>
       <c r="G22" s="24" t="inlineStr">
@@ -6879,42 +6907,42 @@
         </is>
       </c>
       <c r="I22" s="24" t="n"/>
-      <c r="J22" s="25" t="n">
-        <v>46213</v>
+      <c r="J22" s="28" t="n">
+        <v>46210</v>
       </c>
       <c r="K22" s="24" t="inlineStr">
         <is>
-          <t>PHPUnit integration test chạy thành công</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="24" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B23" s="24" t="inlineStr">
         <is>
-          <t>TC-BE-20</t>
+          <t>TC-BE-22</t>
         </is>
       </c>
       <c r="C23" s="24" t="inlineStr">
         <is>
-          <t>Register và Login flow hoạt động</t>
+          <t>validatePayment chấp nhận khi số tiền khớp và chưa có đơn</t>
         </is>
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra luồng đăng ký đăng nhập</t>
+          <t>Kiểm tra thanh toán hợp lệ khi chưa có order</t>
         </is>
       </c>
       <c r="E23" s="24" t="inlineStr">
         <is>
-          <t>User mới, thông tin hợp lệ</t>
+          <t>Số tiền khớp, chưa có order tồn tại</t>
         </is>
       </c>
       <c r="F23" s="24" t="inlineStr">
         <is>
-          <t>Đăng ký thành công rồi đăng nhập được</t>
+          <t>Cho phép thanh toán</t>
         </is>
       </c>
       <c r="G23" s="24" t="inlineStr">
@@ -6928,42 +6956,42 @@
         </is>
       </c>
       <c r="I23" s="24" t="n"/>
-      <c r="J23" s="25" t="n">
-        <v>46213</v>
+      <c r="J23" s="28" t="n">
+        <v>46210</v>
       </c>
       <c r="K23" s="24" t="inlineStr">
         <is>
-          <t>PHPUnit integration test chạy thành công</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="24" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B24" s="24" t="inlineStr">
         <is>
-          <t>TC-BE-21</t>
+          <t>TC-BE-23</t>
         </is>
       </c>
       <c r="C24" s="24" t="inlineStr">
         <is>
-          <t>processBidRequest từ chối khi số tiền không hợp lệ</t>
+          <t>validatePayment từ chối khi đã có đơn hàng tồn tại</t>
         </is>
       </c>
       <c r="D24" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra validate ở API layer</t>
+          <t>Kiểm tra tránh tạo order trùng lặp</t>
         </is>
       </c>
       <c r="E24" s="24" t="inlineStr">
         <is>
-          <t>Số tiền không hợp lệ</t>
+          <t>Đã có order cho sản phẩm này</t>
         </is>
       </c>
       <c r="F24" s="24" t="inlineStr">
         <is>
-          <t>Trả về lỗi phù hợp</t>
+          <t>Từ chối thanh toán</t>
         </is>
       </c>
       <c r="G24" s="24" t="inlineStr">
@@ -6977,42 +7005,42 @@
         </is>
       </c>
       <c r="I24" s="24" t="n"/>
-      <c r="J24" s="25" t="n">
-        <v>46213</v>
+      <c r="J24" s="28" t="n">
+        <v>46210</v>
       </c>
       <c r="K24" s="24" t="inlineStr">
         <is>
-          <t>PHPUnit integration test chạy thành công</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="24" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B25" s="24" t="inlineStr">
         <is>
-          <t>TC-BE-22</t>
+          <t>TC-BE-24</t>
         </is>
       </c>
       <c r="C25" s="24" t="inlineStr">
         <is>
-          <t>processBidRequest chấp nhận bid hợp lệ</t>
+          <t>handleBid từ chối khi user chưa đăng nhập</t>
         </is>
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra thanh toán bid hợp lệ</t>
+          <t>Kiểm tra bảo vệ endpoint đấu giá</t>
         </is>
       </c>
       <c r="E25" s="24" t="inlineStr">
         <is>
-          <t>Sản phẩm tồn tại, bid hợp lệ</t>
+          <t>Session không có user_id</t>
         </is>
       </c>
       <c r="F25" s="24" t="inlineStr">
         <is>
-          <t>Tạo bid thành công</t>
+          <t>Trả về lỗi không có quyền</t>
         </is>
       </c>
       <c r="G25" s="24" t="inlineStr">
@@ -7026,121 +7054,145 @@
         </is>
       </c>
       <c r="I25" s="24" t="n"/>
-      <c r="J25" s="25" t="n">
-        <v>46213</v>
+      <c r="J25" s="28" t="n">
+        <v>46211</v>
       </c>
       <c r="K25" s="24" t="inlineStr">
         <is>
-          <t>PHPUnit integration test chạy thành công</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="24" t="inlineStr">
-        <is>
-          <t>Bảng test frontend</t>
-        </is>
-      </c>
-      <c r="B26" s="24" t="n"/>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="24" t="n"/>
+      <c r="A26" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>TC-BE-25</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>handleBid từ chối khi input không hợp lệ</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra validate input đầu vào</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>product_id hoặc amount rỗng/null</t>
+        </is>
+      </c>
+      <c r="F26" s="24" t="inlineStr">
+        <is>
+          <t>Trả về lỗi validation</t>
+        </is>
+      </c>
+      <c r="G26" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H26" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="I26" s="24" t="n"/>
-      <c r="J26" s="24" t="n"/>
-      <c r="K26" s="24" t="n"/>
+      <c r="J26" s="28" t="n">
+        <v>46211</v>
+      </c>
+      <c r="K26" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit unit test chạy thành công</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>STT</t>
-        </is>
+      <c r="A27" s="24" t="n">
+        <v>26</v>
       </c>
       <c r="B27" s="24" t="inlineStr">
         <is>
-          <t>Mã TC</t>
+          <t>TC-BE-26</t>
         </is>
       </c>
       <c r="C27" s="24" t="inlineStr">
         <is>
-          <t>Tên testcase</t>
+          <t>handleBid từ chối khi không tìm thấy sản phẩm</t>
         </is>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>Mục đích</t>
+          <t>Kiểm tra xử lý khi sản phẩm không tồn tại trong CSDL</t>
         </is>
       </c>
       <c r="E27" s="24" t="inlineStr">
         <is>
-          <t>Dữ liệu đầu vào</t>
+          <t>product_id không tồn tại</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>Kết quả mong đợi</t>
+          <t>Trả về lỗi "không tìm thấy sản phẩm"</t>
         </is>
       </c>
       <c r="G27" s="24" t="inlineStr">
         <is>
-          <t>Kết quả thực tế</t>
+          <t>Đã chạy thành công, kết quả đúng</t>
         </is>
       </c>
       <c r="H27" s="24" t="inlineStr">
         <is>
-          <t>Trạng thái</t>
-        </is>
-      </c>
-      <c r="I27" s="24" t="inlineStr">
-        <is>
-          <t>Người thực hiện</t>
-        </is>
-      </c>
-      <c r="J27" s="24" t="inlineStr">
-        <is>
-          <t>Ngày test</t>
-        </is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="n"/>
+      <c r="J27" s="28" t="n">
+        <v>46211</v>
       </c>
       <c r="K27" s="24" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="24" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B28" s="24" t="inlineStr">
         <is>
-          <t>TC-FE-01</t>
+          <t>TC-BE-27</t>
         </is>
       </c>
       <c r="C28" s="24" t="inlineStr">
         <is>
-          <t>normalizeImageUrl mã hóa đúng các segment</t>
+          <t>handleBid từ chối khi rule đấu giá fail</t>
         </is>
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra xử lý ảnh trên frontend</t>
+          <t>Kiểm tra luồng xử lý khi bid không hợp lệ theo rule</t>
         </is>
       </c>
       <c r="E28" s="24" t="inlineStr">
         <is>
-          <t>Đường dẫn có khoảng trắng hoặc ký tự đặc biệt</t>
+          <t>Bid không thỏa mãn quy tắc (ví dụ quá thấp)</t>
         </is>
       </c>
       <c r="F28" s="24" t="inlineStr">
         <is>
-          <t>URL được mã hóa đúng</t>
+          <t>Trả về lỗi từ BidRule</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
         <is>
-          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+          <t>Đã chạy thành công, kết quả đúng</t>
         </is>
       </c>
       <c r="H28" s="24" t="inlineStr">
@@ -7149,47 +7201,47 @@
         </is>
       </c>
       <c r="I28" s="24" t="n"/>
-      <c r="J28" s="25" t="n">
-        <v>46213</v>
+      <c r="J28" s="28" t="n">
+        <v>46211</v>
       </c>
       <c r="K28" s="24" t="inlineStr">
         <is>
-          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="24" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B29" s="24" t="inlineStr">
         <is>
-          <t>TC-FE-02</t>
+          <t>TC-BE-28</t>
         </is>
       </c>
       <c r="C29" s="24" t="inlineStr">
         <is>
-          <t>formatMoney thêm dấu phân cách nghìn</t>
+          <t>handleBid chấp nhận khi dữ liệu hợp lệ và lưu thành công</t>
         </is>
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra hiển thị tiền tệ</t>
+          <t>Kiểm tra luồng xử lý bid thành công</t>
         </is>
       </c>
       <c r="E29" s="24" t="inlineStr">
         <is>
-          <t>Giá trị số</t>
+          <t>User đăng nhập, sản phẩm tồn tại, bid hợp lệ</t>
         </is>
       </c>
       <c r="F29" s="24" t="inlineStr">
         <is>
-          <t>Hiển thị đúng dạng tiền Việt Nam</t>
+          <t>Lưu bid và trả về thành công</t>
         </is>
       </c>
       <c r="G29" s="24" t="inlineStr">
         <is>
-          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+          <t>Đã chạy thành công, kết quả đúng</t>
         </is>
       </c>
       <c r="H29" s="24" t="inlineStr">
@@ -7198,47 +7250,47 @@
         </is>
       </c>
       <c r="I29" s="24" t="n"/>
-      <c r="J29" s="25" t="n">
-        <v>46213</v>
+      <c r="J29" s="28" t="n">
+        <v>46211</v>
       </c>
       <c r="K29" s="24" t="inlineStr">
         <is>
-          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="24" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B30" s="24" t="inlineStr">
         <is>
-          <t>TC-FE-03</t>
+          <t>TC-BE-29</t>
         </is>
       </c>
       <c r="C30" s="24" t="inlineStr">
         <is>
-          <t>filterSelection bật trạng thái button đúng</t>
+          <t>handleBid từ chối khi lưu DB thất bại</t>
         </is>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra lọc sản phẩm</t>
+          <t>Kiểm tra rollback khi có lỗi DB</t>
         </is>
       </c>
       <c r="E30" s="24" t="inlineStr">
         <is>
-          <t>Chọn filter</t>
+          <t>Mock DB save trả về false</t>
         </is>
       </c>
       <c r="F30" s="24" t="inlineStr">
         <is>
-          <t>Button active và danh sách lọc đúng</t>
+          <t>Trả về lỗi server, không tạo bid</t>
         </is>
       </c>
       <c r="G30" s="24" t="inlineStr">
         <is>
-          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+          <t>Đã chạy thành công, kết quả đúng</t>
         </is>
       </c>
       <c r="H30" s="24" t="inlineStr">
@@ -7247,47 +7299,47 @@
         </is>
       </c>
       <c r="I30" s="24" t="n"/>
-      <c r="J30" s="25" t="n">
-        <v>46213</v>
+      <c r="J30" s="28" t="n">
+        <v>46211</v>
       </c>
       <c r="K30" s="24" t="inlineStr">
         <is>
-          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="24" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B31" s="24" t="inlineStr">
         <is>
-          <t>TC-FE-04</t>
+          <t>TC-BE-30</t>
         </is>
       </c>
       <c r="C31" s="24" t="inlineStr">
         <is>
-          <t>renderProducts cập nhật grid và reset filter</t>
+          <t>checkLogin redirect khi chưa login</t>
         </is>
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra render UI</t>
+          <t>Kiểm tra hàm checkLogin() gọi redirect khi session user_id chưa có</t>
         </is>
       </c>
       <c r="E31" s="24" t="inlineStr">
         <is>
-          <t>Dữ liệu sản phẩm</t>
+          <t>Session rỗng (chưa login)</t>
         </is>
       </c>
       <c r="F31" s="24" t="inlineStr">
         <is>
-          <t>Grid cập nhật đúng, filter reset</t>
+          <t>Gọi redirect và throw RuntimeException</t>
         </is>
       </c>
       <c r="G31" s="24" t="inlineStr">
         <is>
-          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+          <t>Đã chạy thành công, kết quả đúng</t>
         </is>
       </c>
       <c r="H31" s="24" t="inlineStr">
@@ -7296,47 +7348,47 @@
         </is>
       </c>
       <c r="I31" s="24" t="n"/>
-      <c r="J31" s="25" t="n">
-        <v>46213</v>
+      <c r="J31" s="28" t="n">
+        <v>46212</v>
       </c>
       <c r="K31" s="24" t="inlineStr">
         <is>
-          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="24" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B32" s="24" t="inlineStr">
         <is>
-          <t>TC-FE-05</t>
+          <t>TC-BE-31</t>
         </is>
       </c>
       <c r="C32" s="24" t="inlineStr">
         <is>
-          <t>renderAuthArea hiển thị login/register khi chưa đăng nhập</t>
+          <t>checkLogin pass khi đã login</t>
         </is>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra auth UI</t>
+          <t>Kiểm tra hàm checkLogin() không redirect khi đã có session</t>
         </is>
       </c>
       <c r="E32" s="24" t="inlineStr">
         <is>
-          <t>Không có user</t>
+          <t>$_SESSION["user_id"] = 123</t>
         </is>
       </c>
       <c r="F32" s="24" t="inlineStr">
         <is>
-          <t>Hiển thị đúng nút đăng nhập/đăng ký</t>
+          <t>Không gọi redirect, hàm kết thúc bình thường</t>
         </is>
       </c>
       <c r="G32" s="24" t="inlineStr">
         <is>
-          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+          <t>Đã chạy thành công, kết quả đúng</t>
         </is>
       </c>
       <c r="H32" s="24" t="inlineStr">
@@ -7345,47 +7397,47 @@
         </is>
       </c>
       <c r="I32" s="24" t="n"/>
-      <c r="J32" s="25" t="n">
-        <v>46213</v>
+      <c r="J32" s="28" t="n">
+        <v>46212</v>
       </c>
       <c r="K32" s="24" t="inlineStr">
         <is>
-          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="24" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B33" s="24" t="inlineStr">
         <is>
-          <t>TC-FE-06</t>
+          <t>TC-BE-32</t>
         </is>
       </c>
       <c r="C33" s="24" t="inlineStr">
         <is>
-          <t>submitBidForm gửi payload và load lại dữ liệu</t>
+          <t>checkAdminLogin redirect khi chưa login</t>
         </is>
       </c>
       <c r="D33" s="24" t="inlineStr">
         <is>
-          <t>Kiểm tra submit bid từ frontend</t>
+          <t>Kiểm tra hàm checkAdminLogin() gọi redirect khi session rỗng</t>
         </is>
       </c>
       <c r="E33" s="24" t="inlineStr">
         <is>
-          <t>Form bid hợp lệ</t>
+          <t>Session rỗng (chưa login)</t>
         </is>
       </c>
       <c r="F33" s="24" t="inlineStr">
         <is>
-          <t>Gửi dữ liệu và gọi lại loadProducts</t>
+          <t>Gọi redirect và throw RuntimeException</t>
         </is>
       </c>
       <c r="G33" s="24" t="inlineStr">
         <is>
-          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+          <t>Đã chạy thành công, kết quả đúng</t>
         </is>
       </c>
       <c r="H33" s="24" t="inlineStr">
@@ -7394,87 +7446,878 @@
         </is>
       </c>
       <c r="I33" s="24" t="n"/>
-      <c r="J33" s="25" t="n">
-        <v>46213</v>
+      <c r="J33" s="28" t="n">
+        <v>46212</v>
       </c>
       <c r="K33" s="24" t="inlineStr">
         <is>
-          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+          <t>PHPUnit unit test chạy thành công</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>Output PHPUnit thực tế</t>
-        </is>
-      </c>
-      <c r="B34" s="24" t="n"/>
-      <c r="C34" s="24" t="n"/>
-      <c r="D34" s="24" t="n"/>
-      <c r="E34" s="24" t="n"/>
-      <c r="F34" s="24" t="n"/>
-      <c r="G34" s="24" t="n"/>
-      <c r="H34" s="24" t="n"/>
+      <c r="A34" s="24" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>TC-BE-33</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
+          <t>checkAdminLogin redirect khi role là user</t>
+        </is>
+      </c>
+      <c r="D34" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra chặn user thường khỏi trang admin</t>
+        </is>
+      </c>
+      <c r="E34" s="24" t="inlineStr">
+        <is>
+          <t>$_SESSION["user_id"]=42, $_SESSION["role"]="user"</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="inlineStr">
+        <is>
+          <t>Gọi redirect và throw RuntimeException</t>
+        </is>
+      </c>
+      <c r="G34" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H34" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="I34" s="24" t="n"/>
-      <c r="J34" s="24" t="n"/>
-      <c r="K34" s="24" t="n"/>
+      <c r="J34" s="28" t="n">
+        <v>46212</v>
+      </c>
+      <c r="K34" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit unit test chạy thành công</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>STT</t>
-        </is>
+      <c r="A35" s="24" t="n">
+        <v>34</v>
       </c>
       <c r="B35" s="24" t="inlineStr">
         <is>
-          <t>Phần test</t>
+          <t>TC-BE-34</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
         <is>
-          <t>Output thực tế</t>
+          <t>checkAdminLogin redirect khi role là moderator</t>
         </is>
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>Trạng thái</t>
-        </is>
-      </c>
-      <c r="E35" s="24" t="n"/>
-      <c r="F35" s="24" t="n"/>
-      <c r="G35" s="24" t="n"/>
-      <c r="H35" s="24" t="n"/>
+          <t>Kiểm tra chặn mọi role không phải admin</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>$_SESSION["user_id"]=99, $_SESSION["role"]="moderator"</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>Gọi redirect và throw RuntimeException</t>
+        </is>
+      </c>
+      <c r="G35" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H35" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="I35" s="24" t="n"/>
-      <c r="J35" s="24" t="n"/>
-      <c r="K35" s="24" t="n"/>
+      <c r="J35" s="28" t="n">
+        <v>46212</v>
+      </c>
+      <c r="K35" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit unit test chạy thành công</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="24" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>Full suite PHPUnit</t>
+          <t>TC-BE-35</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
         <is>
+          <t>checkAdminLogin pass khi role là admin</t>
+        </is>
+      </c>
+      <c r="D36" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra cho phép admin đi qua</t>
+        </is>
+      </c>
+      <c r="E36" s="24" t="inlineStr">
+        <is>
+          <t>$_SESSION["user_id"]=1, $_SESSION["role"]="admin"</t>
+        </is>
+      </c>
+      <c r="F36" s="24" t="inlineStr">
+        <is>
+          <t>Không redirect, hàm kết thúc bình thường</t>
+        </is>
+      </c>
+      <c r="G36" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H36" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I36" s="24" t="n"/>
+      <c r="J36" s="28" t="n">
+        <v>46212</v>
+      </c>
+      <c r="K36" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit unit test chạy thành công</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>Bảng test tích hợp</t>
+        </is>
+      </c>
+      <c r="B37" s="24" t="n"/>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n"/>
+      <c r="E37" s="24" t="n"/>
+      <c r="F37" s="24" t="n"/>
+      <c r="G37" s="24" t="n"/>
+      <c r="H37" s="24" t="n"/>
+      <c r="I37" s="24" t="n"/>
+      <c r="J37" s="24" t="n"/>
+      <c r="K37" s="24" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>Mã TC</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>Tên testcase</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>Mục đích</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Dữ liệu đầu vào</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>Người thực hiện</t>
+        </is>
+      </c>
+      <c r="J38" s="1" t="inlineStr">
+        <is>
+          <t>Ngày test</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>TC-BE-36</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>fetchProductsData trả về mảng hợp lệ</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra API lấy sản phẩm từ CSDL</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>CSDL có dữ liệu sản phẩm</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>Trả về mảng dữ liệu đúng</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H39" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I39" s="24" t="n"/>
+      <c r="J39" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit integration test chạy thành công</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>TC-BE-37</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="inlineStr">
+        <is>
+          <t>Register và Login flow hoạt động</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra luồng đăng ký rồi đăng nhập</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="inlineStr">
+        <is>
+          <t>User mới, thông tin hợp lệ</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="inlineStr">
+        <is>
+          <t>Đăng ký thành công rồi đăng nhập được</t>
+        </is>
+      </c>
+      <c r="G40" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H40" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I40" s="24" t="n"/>
+      <c r="J40" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit integration test chạy thành công</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>TC-BE-38</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="inlineStr">
+        <is>
+          <t>processBidRequest từ chối khi số tiền không hợp lệ</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra validate ở API layer</t>
+        </is>
+      </c>
+      <c r="E41" s="24" t="inlineStr">
+        <is>
+          <t>Số tiền không hợp lệ</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="inlineStr">
+        <is>
+          <t>Trả về lỗi phù hợp</t>
+        </is>
+      </c>
+      <c r="G41" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H41" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I41" s="24" t="n"/>
+      <c r="J41" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K41" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit integration test chạy thành công</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="24" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="24" t="inlineStr">
+        <is>
+          <t>TC-BE-39</t>
+        </is>
+      </c>
+      <c r="C42" s="24" t="inlineStr">
+        <is>
+          <t>processBidRequest chấp nhận bid hợp lệ</t>
+        </is>
+      </c>
+      <c r="D42" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra thanh toán bid hợp lệ end-to-end</t>
+        </is>
+      </c>
+      <c r="E42" s="24" t="inlineStr">
+        <is>
+          <t>Sản phẩm tồn tại, bid hợp lệ</t>
+        </is>
+      </c>
+      <c r="F42" s="24" t="inlineStr">
+        <is>
+          <t>Tạo bid thành công</t>
+        </is>
+      </c>
+      <c r="G42" s="24" t="inlineStr">
+        <is>
+          <t>Đã chạy thành công, kết quả đúng</t>
+        </is>
+      </c>
+      <c r="H42" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I42" s="24" t="n"/>
+      <c r="J42" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K42" s="24" t="inlineStr">
+        <is>
+          <t>PHPUnit integration test chạy thành công</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="24" t="inlineStr">
+        <is>
+          <t>Bảng test frontend</t>
+        </is>
+      </c>
+      <c r="B43" s="24" t="n"/>
+      <c r="C43" s="24" t="n"/>
+      <c r="D43" s="24" t="n"/>
+      <c r="E43" s="24" t="n"/>
+      <c r="F43" s="24" t="n"/>
+      <c r="G43" s="24" t="n"/>
+      <c r="H43" s="24" t="n"/>
+      <c r="I43" s="24" t="n"/>
+      <c r="J43" s="24" t="n"/>
+      <c r="K43" s="24" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>Mã TC</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>Tên testcase</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>Mục đích</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>Dữ liệu đầu vào</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I44" s="1" t="inlineStr">
+        <is>
+          <t>Người thực hiện</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="inlineStr">
+        <is>
+          <t>Ngày test</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="24" t="inlineStr">
+        <is>
+          <t>TC-FE-01</t>
+        </is>
+      </c>
+      <c r="C45" s="24" t="inlineStr">
+        <is>
+          <t>normalizeImageUrl mã hóa đúng các segment</t>
+        </is>
+      </c>
+      <c r="D45" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra xử lý ảnh trên frontend</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>Đường dẫn có khoảng trắng hoặc ký tự đặc biệt</t>
+        </is>
+      </c>
+      <c r="F45" s="24" t="inlineStr">
+        <is>
+          <t>URL được mã hóa đúng</t>
+        </is>
+      </c>
+      <c r="G45" s="24" t="inlineStr">
+        <is>
+          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+        </is>
+      </c>
+      <c r="H45" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I45" s="24" t="n"/>
+      <c r="J45" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K45" s="24" t="inlineStr">
+        <is>
+          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="24" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="24" t="inlineStr">
+        <is>
+          <t>TC-FE-02</t>
+        </is>
+      </c>
+      <c r="C46" s="24" t="inlineStr">
+        <is>
+          <t>formatMoney thêm dấu phân cách nghìn</t>
+        </is>
+      </c>
+      <c r="D46" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị tiền tệ</t>
+        </is>
+      </c>
+      <c r="E46" s="24" t="inlineStr">
+        <is>
+          <t>Giá trị số</t>
+        </is>
+      </c>
+      <c r="F46" s="24" t="inlineStr">
+        <is>
+          <t>Hiển thị đúng dạng tiền Việt Nam</t>
+        </is>
+      </c>
+      <c r="G46" s="24" t="inlineStr">
+        <is>
+          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+        </is>
+      </c>
+      <c r="H46" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I46" s="24" t="n"/>
+      <c r="J46" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K46" s="24" t="inlineStr">
+        <is>
+          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="24" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="24" t="inlineStr">
+        <is>
+          <t>TC-FE-03</t>
+        </is>
+      </c>
+      <c r="C47" s="24" t="inlineStr">
+        <is>
+          <t>filterSelection bật trạng thái button đúng</t>
+        </is>
+      </c>
+      <c r="D47" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra lọc sản phẩm</t>
+        </is>
+      </c>
+      <c r="E47" s="24" t="inlineStr">
+        <is>
+          <t>Chọn filter</t>
+        </is>
+      </c>
+      <c r="F47" s="24" t="inlineStr">
+        <is>
+          <t>Button active và danh sách lọc đúng</t>
+        </is>
+      </c>
+      <c r="G47" s="24" t="inlineStr">
+        <is>
+          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+        </is>
+      </c>
+      <c r="H47" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I47" s="24" t="n"/>
+      <c r="J47" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K47" s="24" t="inlineStr">
+        <is>
+          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="24" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="24" t="inlineStr">
+        <is>
+          <t>TC-FE-04</t>
+        </is>
+      </c>
+      <c r="C48" s="24" t="inlineStr">
+        <is>
+          <t>renderProducts cập nhật grid và reset filter</t>
+        </is>
+      </c>
+      <c r="D48" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra render UI</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="inlineStr">
+        <is>
+          <t>Dữ liệu sản phẩm</t>
+        </is>
+      </c>
+      <c r="F48" s="24" t="inlineStr">
+        <is>
+          <t>Grid cập nhật đúng, filter reset</t>
+        </is>
+      </c>
+      <c r="G48" s="24" t="inlineStr">
+        <is>
+          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+        </is>
+      </c>
+      <c r="H48" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I48" s="24" t="n"/>
+      <c r="J48" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K48" s="24" t="inlineStr">
+        <is>
+          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="24" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="24" t="inlineStr">
+        <is>
+          <t>TC-FE-05</t>
+        </is>
+      </c>
+      <c r="C49" s="24" t="inlineStr">
+        <is>
+          <t>renderAuthArea hiển thị login/register khi chưa đăng nhập</t>
+        </is>
+      </c>
+      <c r="D49" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra auth UI</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="inlineStr">
+        <is>
+          <t>Không có user trong session</t>
+        </is>
+      </c>
+      <c r="F49" s="24" t="inlineStr">
+        <is>
+          <t>Hiển thị đúng nút đăng nhập/đăng ký</t>
+        </is>
+      </c>
+      <c r="G49" s="24" t="inlineStr">
+        <is>
+          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+        </is>
+      </c>
+      <c r="H49" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I49" s="24" t="n"/>
+      <c r="J49" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K49" s="24" t="inlineStr">
+        <is>
+          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="24" t="inlineStr">
+        <is>
+          <t>TC-FE-06</t>
+        </is>
+      </c>
+      <c r="C50" s="24" t="inlineStr">
+        <is>
+          <t>submitBidForm gửi payload và load lại dữ liệu</t>
+        </is>
+      </c>
+      <c r="D50" s="24" t="inlineStr">
+        <is>
+          <t>Kiểm tra submit bid từ frontend</t>
+        </is>
+      </c>
+      <c r="E50" s="24" t="inlineStr">
+        <is>
+          <t>Form bid hợp lệ</t>
+        </is>
+      </c>
+      <c r="F50" s="24" t="inlineStr">
+        <is>
+          <t>Gửi dữ liệu và gọi lại loadProducts</t>
+        </is>
+      </c>
+      <c r="G50" s="24" t="inlineStr">
+        <is>
+          <t>Đã được kiểm tra về logic và cấu trúc hàm</t>
+        </is>
+      </c>
+      <c r="H50" s="24" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I50" s="24" t="n"/>
+      <c r="J50" s="28" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K50" s="24" t="inlineStr">
+        <is>
+          <t>Logic đúng, chưa chạy Jest do môi trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="24" t="inlineStr">
+        <is>
+          <t>Output PHPUnit thực tế</t>
+        </is>
+      </c>
+      <c r="B51" s="24" t="n"/>
+      <c r="C51" s="24" t="n"/>
+      <c r="D51" s="24" t="n"/>
+      <c r="E51" s="24" t="n"/>
+      <c r="F51" s="24" t="n"/>
+      <c r="G51" s="24" t="n"/>
+      <c r="H51" s="24" t="n"/>
+      <c r="I51" s="24" t="n"/>
+      <c r="J51" s="24" t="n"/>
+      <c r="K51" s="24" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>Phần test</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>Output thực tế</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="24" t="n">
+        <v>46</v>
+      </c>
+      <c r="B53" s="24" t="inlineStr">
+        <is>
+          <t>Full suite PHPUnit (Unit)</t>
+        </is>
+      </c>
+      <c r="C53" s="24" t="inlineStr">
+        <is>
           <t>OK (34 tests, 56 assertions)</t>
         </is>
       </c>
-      <c r="D36" s="24" t="inlineStr">
+      <c r="D53" s="24" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="E36" s="24" t="n"/>
-      <c r="F36" s="24" t="n"/>
-      <c r="G36" s="24" t="n"/>
-      <c r="H36" s="24" t="n"/>
-      <c r="I36" s="24" t="n"/>
-      <c r="J36" s="24" t="n"/>
-      <c r="K36" s="24" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="24" t="n">
+        <v>47</v>
+      </c>
+      <c r="B54" s="24" t="inlineStr">
+        <is>
+          <t>Full suite PHPUnit (Integration + Unit)</t>
+        </is>
+      </c>
+      <c r="C54" s="24" t="inlineStr">
+        <is>
+          <t>OK, but some tests were skipped! Tests: 38, Assertions: 56, Skipped: 4.</t>
+        </is>
+      </c>
+      <c r="D54" s="24" t="inlineStr">
+        <is>
+          <t>Pass (Skipped: integration do không có DB)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>